<commit_message>
Title/abstract and Full-text screening templates
This repository contains standardized templates for title/abstract screening and full-text screening used in our systematic review on physical adversarial attacks. These templates ensure a transparent, consistent, and reproducible screening process in accordance with PRISMA guidelines.
</commit_message>
<xml_diff>
--- a/Screening_Form_Template.xlsx
+++ b/Screening_Form_Template.xlsx
@@ -1,35 +1,259 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375"/>
+    <workbookView windowHeight="17655" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Title and Abstract Screening" sheetId="1" r:id="rId1"/>
+    <sheet name="Full-text Screening" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
+  <si>
+    <t>Title/Abstract Screening Form</t>
+  </si>
+  <si>
+    <t>Reviewer</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>Venue</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t>Topic
+ (Adversarial Attack)</t>
+  </si>
+  <si>
+    <t>Domain 
+( Physical/Real World)</t>
+  </si>
+  <si>
+    <t>Publication Type</t>
+  </si>
+  <si>
+    <t>Publication Quality</t>
+  </si>
+  <si>
+    <t>Language: English?</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Exclusion Reason / Notes</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Li Guojia</t>
+  </si>
+  <si>
+    <t>Li et al.</t>
+  </si>
+  <si>
+    <t>IEEE Transactions on Information Forensics and Security</t>
+  </si>
+  <si>
+    <t>Physical adversarial patch attack for optical fine-grained aircraft recognition</t>
+  </si>
+  <si>
+    <t>Deep neural networks (DNNs) have been widely used in remote sensing but demonstrated to be sensitive with adversarial examples. By introducing carefully designed perturbations to clean images, DNNs can be led to incorrect predictions. Adversarial patch is commonly used to conduct adversarial attack, where traditional methods optimize its content and position separately, neglecting the coupling relation of two factors. In this paper, we propose a black-box attack framework targeting fine-grained aircraft recognition, named PatchGen, simultaneously optimizing both content and position of physical adversarial patches. For the requirements of physical attack, we further constrain the patch in object region and utilize elaborate criteria to evaluate its naturalness to alleviate the distortion when applying the patch in real world. We comprehensively validate our method in fine-grained aircraft classification, extending to object detection subsequently. Extensive experiments demonstrate that the proposed method achieves superior attack performance efficiently for classification and detection tasks in digital domain. Moreover, we validate the effectiveness of the adversarial patch under diverse circumstances in the physical world and prove that our method can be applied to different models as well as various domains.</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Journal</t>
+  </si>
+  <si>
+    <t>top-tier Venue</t>
+  </si>
+  <si>
+    <t>Include</t>
+  </si>
+  <si>
+    <t>Xu Simin</t>
+  </si>
+  <si>
+    <t>Wu et al.</t>
+  </si>
+  <si>
+    <t>arxiv</t>
+  </si>
+  <si>
+    <t>Physical Adversarial Attack on Vehicle Detector in the Carla Simulator</t>
+  </si>
+  <si>
+    <t>In this paper, we tackle the issue of physical adversarial examples for object detectors in the wild. Speciﬁcally, we proposed to generate adversarial patterns to be applied on vehicle surface so that it’s not recognizable by detectors in the photo-realistic Carla simulator. Our approach contains two main techniques, an Enlarge-and-Repeat process and a Discrete Searching method, to craft mosaic-like adversarial vehicle textures without access to neither the model weight of the detector nor a diﬀerential rendering procedure. The experimental results demonstrate the eﬀectiveness of our approach in the simulator.</t>
+  </si>
+  <si>
+    <t>Preprint</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Exclude</t>
+  </si>
+  <si>
+    <t>Non-peer-reviewed</t>
+  </si>
+  <si>
+    <t>Full-text Screening</t>
+  </si>
+  <si>
+    <t>Exclusion Criterion</t>
+  </si>
+  <si>
+    <t>Sato et al.</t>
+  </si>
+  <si>
+    <t>Invisible Reflections: Leveraging Infrared Laser Reflections to Target Traffic Sign Perception</t>
+  </si>
+  <si>
+    <t>Network and Distributed System Security Symposium</t>
+  </si>
+  <si>
+    <t>Cheng et al.</t>
+  </si>
+  <si>
+    <t>Physical Attack on Monocular Depth Estimation with Optimal Adversarial Patches</t>
+  </si>
+  <si>
+    <t>European Conference on Computer Vision</t>
+  </si>
+  <si>
+    <t>C2: Non-vision tasks</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.25"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11.25"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16.5"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -176,7 +400,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -185,6 +409,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -370,12 +606,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -496,139 +747,208 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -689,6 +1009,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
+<customStorage xmlns="https://web.wps.cn/et/2018/main">
+  <book/>
+  <sheets/>
+</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -941,9 +1268,228 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="50" customHeight="1" outlineLevelRow="4"/>
+  <cols>
+    <col min="1" max="5" width="14.875" customWidth="1"/>
+    <col min="6" max="6" width="34.375" customWidth="1"/>
+    <col min="7" max="7" width="62.125" customWidth="1"/>
+    <col min="8" max="14" width="18.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" customHeight="1" spans="1:14">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+    </row>
+    <row r="2" s="17" customFormat="1" customHeight="1" spans="1:14">
+      <c r="A2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" s="18" customFormat="1" customHeight="1" spans="1:14">
+      <c r="A3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="M3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" s="4" customFormat="1" customHeight="1" spans="1:14">
+      <c r="A4" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="22">
+        <v>45840</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="15">
+        <v>2025</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="23"/>
+    </row>
+    <row r="5" s="4" customFormat="1" customHeight="1" spans="1:14">
+      <c r="A5" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="22">
+        <v>45848</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="15">
+        <v>2020</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L5" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5" s="21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:I1 L1 L4:L1048576 H4:I1048576">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1 J4:J1048576">
+      <formula1>"Conference, Journal, Preprint, other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 M4:M1048576">
+      <formula1>"Include,Exclude"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1 N4:N1048576">
+      <formula1>"Non-Relevance,Non-peer-reviewed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K2 K4:K1048576">
+      <formula1>"CORE A /B,Scimago Q1/Q2, top-tier Venue,Other Peer-Reviewed,Unknown"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
@@ -953,9 +1499,117 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelRow="4" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="3" width="18.125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="45.125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.875" style="3" customWidth="1"/>
+    <col min="6" max="8" width="26.5" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" customHeight="1" spans="1:7">
+      <c r="A1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+    </row>
+    <row r="2" s="1" customFormat="1" customHeight="1" spans="1:8">
+      <c r="A2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" customHeight="1" spans="1:7">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="12">
+        <v>45868</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="15">
+        <v>2024</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:8">
+      <c r="A4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="12">
+        <v>45869</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="15">
+        <v>2020</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="5:5">
+      <c r="E5" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1 G3:G1048576">
+      <formula1>"Include,Exclude"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 H3:H1048576">
+      <formula1>"C1:Non-physical deployment,C2: Non-vision tasks,C3: Lack of cohesive contribution"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>